<commit_message>
added apply job,view job & run ai screening
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -417,11 +417,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -484,27 +484,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>resume_1.txt</t>
+          <t>resume_31.pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>86.11000061035156</v>
+        <v>73.30000305175781</v>
       </c>
       <c r="D2" t="n">
         <v>60</v>
       </c>
       <c r="E2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F2" t="n">
         <v>75</v>
       </c>
-      <c r="F2" t="n">
-        <v>50</v>
-      </c>
       <c r="G2" t="n">
-        <v>72.44000244140625</v>
+        <v>74.81999969482422</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>python, aws, docker, kubernetes</t>
+          <t>kubernetes, aws, python, docker</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -515,11 +515,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>resume_3.txt</t>
+          <t>resume_1.txt</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>49.47999954223633</v>
+        <v>86.11000061035156</v>
       </c>
       <c r="D3" t="n">
         <v>60</v>
@@ -528,21 +528,17 @@
         <v>75</v>
       </c>
       <c r="F3" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="G3" t="n">
-        <v>60.29000091552734</v>
+        <v>72.44000244140625</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>python</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>aws, docker, kubernetes</t>
-        </is>
-      </c>
+          <t>kubernetes, aws, python, docker</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -550,63 +546,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>resume_4.txt</t>
+          <t>resume_6.txt</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>48.66999816894531</v>
+        <v>35.40000152587891</v>
       </c>
       <c r="D4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>100</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>56.47000122070312</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>python, aws</t>
-        </is>
-      </c>
+        <v>36.65999984741211</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>docker, kubernetes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>resume_5.txt</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>36.70999908447266</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>75</v>
-      </c>
-      <c r="F5" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" t="n">
-        <v>34.68999862670898</v>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>python, aws, docker, kubernetes</t>
+          <t>kubernetes, docker, aws, python</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added phone no ,gmail,name column
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>73.30000305175781</v>
+        <v>73.3</v>
       </c>
       <c r="D2" t="n">
         <v>60</v>
@@ -500,11 +500,11 @@
         <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>74.81999969482422</v>
+        <v>74.81999999999999</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>kubernetes, aws, python, docker</t>
+          <t>python, aws, docker, kubernetes</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -519,7 +519,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>86.11000061035156</v>
+        <v>86.11</v>
       </c>
       <c r="D3" t="n">
         <v>60</v>
@@ -531,11 +531,11 @@
         <v>50</v>
       </c>
       <c r="G3" t="n">
-        <v>72.44000244140625</v>
+        <v>72.44</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>kubernetes, aws, python, docker</t>
+          <t>python, aws, docker, kubernetes</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35.40000152587891</v>
+        <v>35.4</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -562,12 +562,12 @@
         <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>36.65999984741211</v>
+        <v>36.66</v>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>kubernetes, docker, aws, python</t>
+          <t>python, aws, docker, kubernetes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added applied button & fix bug
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -417,21 +417,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="41" customWidth="1" min="10" max="10"/>
-    <col width="71" customWidth="1" min="11" max="11"/>
-    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,14 +484,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>resume_18.txt</t>
+          <t>1774456397_resume_1.txt</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>44.5</v>
+        <v>86.11</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E2" t="n">
         <v>75</v>
@@ -503,27 +500,47 @@
         <v>50</v>
       </c>
       <c r="G2" t="n">
-        <v>37.8</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>aws, python, kubernetes, docker</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>L, i, a, m,  , T, h, o, m, p, s, o, n</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>l, i, a, m, ., t, h, o, m, p, s, o, n, @, e, m, a, i, l, ., c, o, m</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N, o, t,  , F, o, u, n, d</t>
+        <v>72.44</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>aws, python, docker, kubernetes</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1774456460_resume_4.txt</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>48.67</v>
+      </c>
+      <c r="D3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" t="n">
+        <v>56.47</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>aws, python</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>kubernetes, docker</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated db config for deployment
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -417,18 +417,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,63 +484,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1774456397_resume_1.txt</t>
+          <t>SUSHIL RK_DA.pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>86.11</v>
+        <v>35.4</v>
       </c>
       <c r="D2" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="F2" t="n">
         <v>50</v>
       </c>
       <c r="G2" t="n">
-        <v>72.44</v>
+        <v>30.16</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>aws, python, docker, kubernetes</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1774456460_resume_4.txt</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>48.67</v>
-      </c>
-      <c r="D3" t="n">
-        <v>40</v>
-      </c>
-      <c r="E3" t="n">
-        <v>100</v>
-      </c>
-      <c r="F3" t="n">
-        <v>50</v>
-      </c>
-      <c r="G3" t="n">
-        <v>56.47</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>aws, python</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>kubernetes, docker</t>
+          <t>python, pandas</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>sql, machine learning, tensorflow</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix float32 json error
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>73.3</v>
+        <v>74.48</v>
       </c>
       <c r="D2" t="n">
         <v>60</v>
@@ -500,11 +500,11 @@
         <v>75</v>
       </c>
       <c r="G2" t="n">
-        <v>74.81999999999999</v>
+        <v>75.29000000000001</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>python, kubernetes, docker, aws</t>
+          <t>docker, python, kubernetes, aws</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>

</xml_diff>

<commit_message>
added TF-IDF + Cosine Similarity
</commit_message>
<xml_diff>
--- a/AI_Resume_Ranking_Report.xlsx
+++ b/AI_Resume_Ranking_Report.xlsx
@@ -417,18 +417,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="41" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="49" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -449,30 +450,35 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>TF-IDF Score</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Skill Score</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Experience Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Education Score</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Final Score</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Matched Skills</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Missing Skills</t>
         </is>
@@ -484,30 +490,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1780942564_ROHAN KULKARNI  resume.pdf</t>
+          <t>1781203020_NEHA DESHMUKH  resume.pdf</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>68.20999999999999</v>
+        <v>51.99</v>
       </c>
       <c r="D2" t="n">
+        <v>22.63</v>
+      </c>
+      <c r="E2" t="n">
         <v>60</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>25</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>50</v>
       </c>
-      <c r="G2" t="n">
-        <v>55.28</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>python, aws, kubernetes, docker</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>41.89</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>pytorch, tensorflow, machine learning, python</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>docker, sql</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -515,32 +528,35 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1780942662_VIKRAM SINGH resume.pdf</t>
+          <t>1781203140_SNEHA NAIR resume.pdf</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>36.58</v>
+        <v>43.25</v>
       </c>
       <c r="D3" t="n">
-        <v>80</v>
+        <v>16.63</v>
       </c>
       <c r="E3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F3" t="n">
         <v>25</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>50</v>
       </c>
-      <c r="G3" t="n">
-        <v>48.63</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>python, aws, docker</t>
-        </is>
+      <c r="H3" t="n">
+        <v>37.47</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>kubernetes</t>
+          <t>tensorflow, sql, machine learning, python</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>pytorch, docker</t>
         </is>
       </c>
     </row>
@@ -550,32 +566,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1780942371_NEHA DESHMUKH  resume.pdf</t>
+          <t>1781203309_ROHAN KULKARNI  resume.pdf</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>41.9</v>
+        <v>48.15</v>
       </c>
       <c r="D4" t="n">
+        <v>10.93</v>
+      </c>
+      <c r="E4" t="n">
         <v>60</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>25</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>50</v>
       </c>
-      <c r="G4" t="n">
-        <v>44.76</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>python, aws</t>
-        </is>
+      <c r="H4" t="n">
+        <v>37.23</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>kubernetes, docker</t>
+          <t>docker, python</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>pytorch, tensorflow, sql, machine learning</t>
         </is>
       </c>
     </row>
@@ -585,32 +604,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1780942519_Rahul Sharma resume.pdf</t>
+          <t>1781202824_VIKRAM SINGH resume.pdf</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>39.26</v>
+        <v>38.8</v>
       </c>
       <c r="D5" t="n">
-        <v>60</v>
+        <v>6.25</v>
       </c>
       <c r="E5" t="n">
+        <v>80</v>
+      </c>
+      <c r="F5" t="n">
         <v>25</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>50</v>
       </c>
-      <c r="G5" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>python, aws</t>
-        </is>
+      <c r="H5" t="n">
+        <v>37.02</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>kubernetes, docker</t>
+          <t>docker, python, sql</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>pytorch, tensorflow, machine learning</t>
         </is>
       </c>
     </row>
@@ -620,32 +642,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1780942196_AMIT VERMA resume.pdf</t>
+          <t>1781203059_PRIYA PATIL resume.pdf</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>35.86</v>
+        <v>40.94</v>
       </c>
       <c r="D6" t="n">
+        <v>14.95</v>
+      </c>
+      <c r="E6" t="n">
         <v>60</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>25</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>50</v>
       </c>
-      <c r="G6" t="n">
-        <v>42.34</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>python, docker</t>
-        </is>
+      <c r="H6" t="n">
+        <v>36.27</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>aws, kubernetes</t>
+          <t>python, sql, machine learning</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>pytorch, docker, tensorflow</t>
         </is>
       </c>
     </row>
@@ -655,32 +680,35 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1780942620_SNEHA NAIR resume.pdf</t>
+          <t>1781203096_Rahul Sharma resume.pdf</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>29.44</v>
+        <v>38.52</v>
       </c>
       <c r="D7" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="E7" t="n">
         <v>60</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>25</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>50</v>
       </c>
-      <c r="G7" t="n">
-        <v>39.78</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
+      <c r="H7" t="n">
+        <v>32.99</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>aws, kubernetes, docker</t>
+          <t>python, sql</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>pytorch, docker, tensorflow, machine learning</t>
         </is>
       </c>
     </row>
@@ -690,32 +718,35 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1780942431_PRIYA PATIL resume.pdf</t>
+          <t>1781202869_AMIT VERMA resume.pdf</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>26.42</v>
+        <v>31.94</v>
       </c>
       <c r="D8" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="E8" t="n">
         <v>60</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>25</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>50</v>
       </c>
-      <c r="G8" t="n">
-        <v>38.57</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>python</t>
-        </is>
+      <c r="H8" t="n">
+        <v>31.03</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>aws, kubernetes, docker</t>
+          <t>docker, python, sql</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>pytorch, tensorflow, machine learning</t>
         </is>
       </c>
     </row>
@@ -725,32 +756,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1780942258_ARJUN MEHTA  resume.pdf</t>
+          <t>1781202944_ARJUN MEHTA  resume.pdf</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>40.05</v>
+        <v>39.58</v>
       </c>
       <c r="D9" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="E9" t="n">
         <v>40</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>25</v>
       </c>
-      <c r="F9" t="n">
+      <c r="G9" t="n">
         <v>50</v>
       </c>
-      <c r="G9" t="n">
-        <v>38.02</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>python, aws</t>
-        </is>
+      <c r="H9" t="n">
+        <v>28.02</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>kubernetes, docker</t>
+          <t>python</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>pytorch, tensorflow, docker, sql, machine learning</t>
         </is>
       </c>
     </row>
@@ -760,28 +794,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>1780942323_KAVYA JOSHI  resume.pdf</t>
+          <t>1781202986_KAVYA JOSHI  resume.pdf</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>19.84</v>
+        <v>20.15</v>
       </c>
       <c r="D10" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="E10" t="n">
         <v>0</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>25</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>50</v>
       </c>
-      <c r="G10" t="n">
-        <v>17.94</v>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>python, aws, kubernetes, docker</t>
+      <c r="H10" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>pytorch, docker, tensorflow, python, sql, machine learning</t>
         </is>
       </c>
     </row>

</xml_diff>